<commit_message>
added cases to dummy_traject
</commit_message>
<xml_diff>
--- a/scripts/example_input/dummy_traject/16-X_000/16-X_000_DP000-DP003_1.xlsx
+++ b/scripts/example_input/dummy_traject/16-X_000/16-X_000_DP000-DP003_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKA\sources\github\faalkansbeheer\scripts\example_input\dummy_traject\16-X_000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D19639-4BA9-4E24-8D68-F55D9AB373C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6A63CD-AC9E-43DB-950B-B1FAB729B603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37215" yWindow="9000" windowWidth="27105" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38505" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario1" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
   <si>
     <t>Template:</t>
   </si>
@@ -206,10 +206,13 @@
     <t>Glijvlak met reststerkte</t>
   </si>
   <si>
-    <t>Overstroming</t>
-  </si>
-  <si>
     <t>Vervolgmechanismen</t>
+  </si>
+  <si>
+    <t>Overstroming | glijvlak zonder reststerkte</t>
+  </si>
+  <si>
+    <t>Overstroming | glijvlak met reststerkte</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>1</v>
       </c>
@@ -1221,7 +1224,7 @@
         <v>47</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -1230,7 +1233,7 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
     </row>
-    <row r="14" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>2</v>
       </c>
@@ -1244,10 +1247,10 @@
         <v>48</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1466,16 +1469,16 @@
       <c r="D29">
         <v>5.9026000000000014</v>
       </c>
-      <c r="E29">
-        <v>6.6807201268858071E-2</v>
-      </c>
-      <c r="G29" t="str">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H29" s="13">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v>1.4999999999999998</v>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v>2.2750131948179191E-2</v>
+      </c>
+      <c r="H29" s="13" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1492,16 +1495,16 @@
       <c r="D30">
         <v>6.65</v>
       </c>
-      <c r="E30">
-        <v>0.1586552539314571</v>
-      </c>
-      <c r="G30" t="str">
-        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H30" s="13">
-        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v>1.0000000000000013</v>
+      <c r="F30">
+        <v>1.5</v>
+      </c>
+      <c r="G30">
+        <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
+        <v>6.6807201268858057E-2</v>
+      </c>
+      <c r="H30" s="13" t="str">
+        <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1513,7 +1516,7 @@
       </c>
       <c r="C31" t="str">
         <f t="array" ref="C31">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming</v>
+        <v>Overstroming | glijvlak zonder reststerkte</v>
       </c>
       <c r="D31">
         <v>3</v>
@@ -1539,7 +1542,7 @@
       </c>
       <c r="C32" t="str">
         <f t="array" ref="C32">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming</v>
+        <v>Overstroming | glijvlak zonder reststerkte</v>
       </c>
       <c r="D32">
         <v>7</v>
@@ -1597,7 +1600,7 @@
         <v>6.65</v>
       </c>
       <c r="E34">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="G34" t="str">
         <f>IF(FCPunten[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten[[#This Row],[Beta_h]],TRUE))</f>
@@ -1605,7 +1608,7 @@
       </c>
       <c r="H34" s="13">
         <f>IF(FCPunten[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten[[#This Row],[Pf_h]]))</f>
-        <v>1.0364333894937898</v>
+        <v>1.2815515655446006</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1669,7 +1672,7 @@
       </c>
       <c r="C37" t="str">
         <f t="array" ref="C37">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming</v>
+        <v>Overstroming | glijvlak met reststerkte</v>
       </c>
       <c r="D37">
         <v>4.4000000000000004</v>
@@ -1695,7 +1698,7 @@
       </c>
       <c r="C38" t="str">
         <f t="array" ref="C38">IF(SUM(FCPunten[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten[[#This Row],[Faalpad_ID]],FCPunten[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming</v>
+        <v>Overstroming | glijvlak met reststerkte</v>
       </c>
       <c r="D38">
         <v>6.65</v>
@@ -2158,65 +2161,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document CB" ma:contentTypeID="0x010100A075C07AB76F2344B407AD577D6B92360100C7929242D85FED4E837C6D4097594A04" ma:contentTypeVersion="17" ma:contentTypeDescription="WSRL Document CB" ma:contentTypeScope="" ma:versionID="18c34f52c90103a5ca6273d5693675c9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="338e11dd-9b15-475b-8471-fcb79439c886" xmlns:ns3="edfbc03d-db26-4301-8719-99148ee26221" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b0dc2be265e99dcf2e366001e246f12" ns2:_="" ns3:_="">
     <xsd:import namespace="338e11dd-9b15-475b-8471-fcb79439c886"/>
@@ -2498,6 +2442,65 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{633EBDFC-B21A-4048-98F2-0CE0F24CB488}">
   <ds:schemaRefs>
@@ -2510,22 +2513,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{263B6D11-DEF0-4FE0-9C65-6A39ECB04A89}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB6BAA4-1CD2-494A-9433-1FC41C42B0F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC89D3C9-3D59-4FE5-907B-98550F7D511D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2542,4 +2529,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB6BAA4-1CD2-494A-9433-1FC41C42B0F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{263B6D11-DEF0-4FE0-9C65-6A39ECB04A89}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>